<commit_message>
Adicionado uma nova categoria para a planilha, pequena mudança na ordem dos botões, otimização do prompt da IA
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I33"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -462,6 +462,11 @@
           <t>Aporte Mensal</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Categoria</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -495,6 +500,7 @@
       <c r="I2" t="n">
         <v>400</v>
       </c>
+      <c r="J2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -524,6 +530,7 @@
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -553,6 +560,7 @@
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -582,6 +590,7 @@
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -607,6 +616,7 @@
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -632,6 +642,7 @@
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr"/>
+      <c r="J7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -657,6 +668,7 @@
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr"/>
+      <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -682,6 +694,7 @@
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -711,6 +724,7 @@
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -736,6 +750,7 @@
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -765,6 +780,7 @@
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -790,6 +806,7 @@
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -815,6 +832,7 @@
       <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -844,6 +862,7 @@
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -869,6 +888,7 @@
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -898,6 +918,7 @@
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -923,6 +944,7 @@
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -948,6 +970,7 @@
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -973,6 +996,7 @@
       <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1002,6 +1026,7 @@
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1027,6 +1052,7 @@
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1056,6 +1082,7 @@
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1085,6 +1112,7 @@
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1110,6 +1138,7 @@
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1135,6 +1164,7 @@
       <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1160,6 +1190,7 @@
       <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1185,6 +1216,7 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1214,6 +1246,7 @@
       <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1243,6 +1276,7 @@
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1268,6 +1302,7 @@
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1293,6 +1328,7 @@
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1318,6 +1354,71 @@
       <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Videogame</t>
+        </is>
+      </c>
+      <c r="C34" t="n">
+        <v>50</v>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Saída</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Lazer</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>25/10/2026</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Conta de Luz</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>200</v>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Conta</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>10/11/2026</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr"/>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Contas de Casa</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>